<commit_message>
feat: implement 2-up layout for 32x25 label
</commit_message>
<xml_diff>
--- a/DUKAN BAI STICKER.xlsx
+++ b/DUKAN BAI STICKER.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="85">
   <si>
     <t>PRODUCT NAME</t>
   </si>
@@ -264,13 +264,25 @@
   </si>
   <si>
     <t>mustard seeds</t>
+  </si>
+  <si>
+    <t>RAJWADI GARAM MASALA</t>
+  </si>
+  <si>
+    <t>RGM-1026</t>
+  </si>
+  <si>
+    <t>100 gm- 120  , 250 gms- 300 , 500 gms- 600   , 1 kg- 1200</t>
+  </si>
+  <si>
+    <t>(In Descending Order By weight) Coriander, Chilli, Edible Common Salt, Cumin, Fennel, Cassia Bark, Star Anise, Black Cardamom, Bay Leaf, Caraway, Sichuan Pepper, Black Pepper,Clove, Cotton seed oil, Mace.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -299,6 +311,20 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -320,7 +346,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -343,11 +369,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -367,6 +408,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1166,6 +1209,21 @@
         <v>80</v>
       </c>
     </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="B31" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C31" s="9"/>
+      <c r="D31" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="F31" s="10" t="s">
+        <v>84</v>
+      </c>
+    </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>68</v>
@@ -1179,6 +1237,7 @@
     <mergeCell ref="A1:D3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>